<commit_message>
updated ccamc, crpunl, ttle
</commit_message>
<xml_diff>
--- a/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
+++ b/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\US\Models\eps-us\InputData\elec\CRpUNL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\AR\elec\CRpUNL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FDBFBA6-B529-49A7-A4EF-4EC1C6ADD991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAAE3D70-309F-4339-AC4B-303594F96C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23640" xr2:uid="{67B50A2A-83E2-40E1-A966-DC033ADD8EBF}"/>
+    <workbookView xWindow="7860" yWindow="420" windowWidth="20940" windowHeight="16860" xr2:uid="{67B50A2A-83E2-40E1-A966-DC033ADD8EBF}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -133,6 +133,15 @@
   </si>
   <si>
     <t>CRpUNL Capacity Retired per Unit Net Loss</t>
+  </si>
+  <si>
+    <t>Hydro plants typically have other revenue streams and other considerations when determining whether or not to retire them,</t>
+  </si>
+  <si>
+    <t>so we assume a value of zero</t>
+  </si>
+  <si>
+    <t>Arkansas</t>
   </si>
 </sst>
 </file>
@@ -171,12 +180,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -191,13 +206,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,15 +529,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B7A547-DAFD-4CBC-90C6-A86A1413C282}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="5">
+        <v>45303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -528,24 +551,34 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -608,8 +641,8 @@
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>159.27199999999999</v>
+      <c r="B6" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -688,7 +721,7 @@
       <c r="A16" t="s">
         <v>17</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="4">
         <v>0</v>
       </c>
     </row>
@@ -696,7 +729,7 @@
       <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="4">
         <v>0</v>
       </c>
     </row>
@@ -712,7 +745,7 @@
       <c r="A19" t="s">
         <v>21</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="4">
         <v>0</v>
       </c>
     </row>
@@ -720,7 +753,7 @@
       <c r="A20" t="s">
         <v>22</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="4">
         <v>0</v>
       </c>
     </row>
@@ -728,7 +761,7 @@
       <c r="A21" t="s">
         <v>23</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="4">
         <v>0</v>
       </c>
     </row>
@@ -736,7 +769,7 @@
       <c r="A22" t="s">
         <v>24</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="4">
         <v>0</v>
       </c>
     </row>
@@ -744,7 +777,7 @@
       <c r="A23" t="s">
         <v>25</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="4">
         <v>0</v>
       </c>
     </row>
@@ -752,7 +785,7 @@
       <c r="A24" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="4">
         <v>0</v>
       </c>
     </row>
@@ -760,7 +793,7 @@
       <c r="A25" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>